<commit_message>
feat: replace broken links and add diverse learning resources
</commit_message>
<xml_diff>
--- a/dataset/GuidanceDataset.xlsx
+++ b/dataset/GuidanceDataset.xlsx
@@ -796,7 +796,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I41"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -954,10 +954,10 @@
         <v>Introduction to Law</v>
       </c>
       <c r="D6" t="str">
-        <v>OpenLearn</v>
+        <v>Coursera</v>
       </c>
       <c r="E6" t="str">
-        <v>https://www.open.edu/openlearn/society-politics-law/law</v>
+        <v>https://www.coursera.org/learn/law-student</v>
       </c>
       <c r="F6" t="str">
         <v>Course</v>
@@ -969,7 +969,7 @@
         <v>Free</v>
       </c>
       <c r="I6" t="str">
-        <v/>
+        <v>14 hours</v>
       </c>
     </row>
     <row r="7">
@@ -980,13 +980,13 @@
         <v>S014</v>
       </c>
       <c r="C7" t="str">
-        <v>Data Analysis in Business</v>
+        <v>Qualitative Research Methods</v>
       </c>
       <c r="D7" t="str">
-        <v>OpenLearn</v>
+        <v>Coursera</v>
       </c>
       <c r="E7" t="str">
-        <v>https://www.open.edu/openlearn/money-business/qualitative-data-analysis</v>
+        <v>https://www.coursera.org/learn/qualitative-research</v>
       </c>
       <c r="F7" t="str">
         <v>Course</v>
@@ -998,7 +998,7 @@
         <v>Free</v>
       </c>
       <c r="I7" t="str">
-        <v>10 hours</v>
+        <v>18 hours</v>
       </c>
     </row>
     <row r="8">
@@ -1009,13 +1009,13 @@
         <v>S015</v>
       </c>
       <c r="C8" t="str">
-        <v>Conflict Resolution</v>
+        <v>Conflict Resolution Skills</v>
       </c>
       <c r="D8" t="str">
-        <v>OpenLearn</v>
+        <v>Coursera</v>
       </c>
       <c r="E8" t="str">
-        <v>https://www.open.edu/openlearn/money-business/leadership-management/conflict-resolution</v>
+        <v>https://www.coursera.org/learn/conflict-resolution-skills</v>
       </c>
       <c r="F8" t="str">
         <v>Course</v>
@@ -1027,7 +1027,7 @@
         <v>Free</v>
       </c>
       <c r="I8" t="str">
-        <v>6 hours</v>
+        <v>12 hours</v>
       </c>
     </row>
     <row r="9">
@@ -1038,25 +1038,25 @@
         <v>S001</v>
       </c>
       <c r="C9" t="str">
-        <v>Effective Communication</v>
+        <v>Communication Skills Courses</v>
       </c>
       <c r="D9" t="str">
-        <v>OpenLearn</v>
+        <v>Coursera</v>
       </c>
       <c r="E9" t="str">
-        <v>https://www.open.edu/openlearn/money-business/leadership-management/effective-communication-the-workplace</v>
+        <v>https://www.coursera.org/courses?query=communication</v>
       </c>
       <c r="F9" t="str">
-        <v>Course</v>
+        <v>Course Catalog</v>
       </c>
       <c r="G9" t="str">
-        <v>Beginner</v>
+        <v>Mixed</v>
       </c>
       <c r="H9" t="str">
-        <v>Free</v>
+        <v>Mixed</v>
       </c>
       <c r="I9" t="str">
-        <v>12 hours</v>
+        <v>Variable</v>
       </c>
     </row>
     <row r="10">
@@ -1070,10 +1070,10 @@
         <v>Critical Thinking Skills</v>
       </c>
       <c r="D10" t="str">
-        <v>OpenLearn</v>
+        <v>Coursera</v>
       </c>
       <c r="E10" t="str">
-        <v>https://www.open.edu/openlearn/money-business/leadership-management/critical-thinking</v>
+        <v>https://www.coursera.org/learn/critical-thinking-skills</v>
       </c>
       <c r="F10" t="str">
         <v>Course</v>
@@ -1096,25 +1096,25 @@
         <v>S003</v>
       </c>
       <c r="C11" t="str">
-        <v>Leadership and Followership</v>
+        <v>Leadership Courses</v>
       </c>
       <c r="D11" t="str">
-        <v>OpenLearn</v>
+        <v>Coursera</v>
       </c>
       <c r="E11" t="str">
-        <v>https://www.open.edu/openlearn/money-business/leadership-management/leadership-and-followership</v>
+        <v>https://www.coursera.org/courses?query=leadership</v>
       </c>
       <c r="F11" t="str">
-        <v>Course</v>
+        <v>Course Catalog</v>
       </c>
       <c r="G11" t="str">
-        <v>Intermediate</v>
+        <v>Mixed</v>
       </c>
       <c r="H11" t="str">
-        <v>Free</v>
+        <v>Mixed</v>
       </c>
       <c r="I11" t="str">
-        <v>8 hours</v>
+        <v>Variable</v>
       </c>
     </row>
     <row r="12">
@@ -1125,13 +1125,13 @@
         <v>S006</v>
       </c>
       <c r="C12" t="str">
-        <v>Learning to Teach, Learning to Speak</v>
+        <v>Introduction to Public Speaking</v>
       </c>
       <c r="D12" t="str">
-        <v>OpenLearn</v>
+        <v>Coursera</v>
       </c>
       <c r="E12" t="str">
-        <v>https://www.open.edu/openlearn/education-development/learning-teach-learning-speak</v>
+        <v>https://www.coursera.org/learn/public-speaking</v>
       </c>
       <c r="F12" t="str">
         <v>Course</v>
@@ -1143,7 +1143,7 @@
         <v>Free</v>
       </c>
       <c r="I12" t="str">
-        <v>4 hours</v>
+        <v>12 hours</v>
       </c>
     </row>
     <row r="13">
@@ -1154,13 +1154,13 @@
         <v>S007</v>
       </c>
       <c r="C13" t="str">
-        <v>Understanding Health and Social Care Research</v>
+        <v>Understanding Research Methods</v>
       </c>
       <c r="D13" t="str">
-        <v>OpenLearn</v>
+        <v>Coursera</v>
       </c>
       <c r="E13" t="str">
-        <v>https://www.open.edu/openlearn/health-sports-psychology/health/understanding-health-and-social-care-research</v>
+        <v>https://www.coursera.org/learn/research-methods</v>
       </c>
       <c r="F13" t="str">
         <v>Course</v>
@@ -1172,7 +1172,7 @@
         <v>Free</v>
       </c>
       <c r="I13" t="str">
-        <v>15 hours</v>
+        <v>20 hours</v>
       </c>
     </row>
     <row r="14">
@@ -1183,13 +1183,13 @@
         <v>S008</v>
       </c>
       <c r="C14" t="str">
-        <v>Problem Solving and Decision Making</v>
+        <v>Effective Problem-Solving and Decision-Making</v>
       </c>
       <c r="D14" t="str">
-        <v>OpenLearn</v>
+        <v>Coursera</v>
       </c>
       <c r="E14" t="str">
-        <v>https://www.open.edu/openlearn/money-business/leadership-management/problem-solving-and-decision-making</v>
+        <v>https://www.coursera.org/learn/problem-solving</v>
       </c>
       <c r="F14" t="str">
         <v>Course</v>
@@ -1201,7 +1201,7 @@
         <v>Free</v>
       </c>
       <c r="I14" t="str">
-        <v>12 hours</v>
+        <v>15 hours</v>
       </c>
     </row>
     <row r="15">
@@ -1212,13 +1212,13 @@
         <v>S009</v>
       </c>
       <c r="C15" t="str">
-        <v>Working in Teams</v>
+        <v>Teamwork Skills: Communicating Effectively in Groups</v>
       </c>
       <c r="D15" t="str">
-        <v>OpenLearn</v>
+        <v>Coursera</v>
       </c>
       <c r="E15" t="str">
-        <v>https://www.open.edu/openlearn/money-business/leadership-management/working-teams</v>
+        <v>https://www.coursera.org/learn/teamwork-skills-effective-communication</v>
       </c>
       <c r="F15" t="str">
         <v>Course</v>
@@ -1230,7 +1230,7 @@
         <v>Free</v>
       </c>
       <c r="I15" t="str">
-        <v>15 hours</v>
+        <v>10 hours</v>
       </c>
     </row>
     <row r="16">
@@ -1241,13 +1241,13 @@
         <v>S010</v>
       </c>
       <c r="C16" t="str">
-        <v>English: Skills for Learning</v>
+        <v>Business Writing</v>
       </c>
       <c r="D16" t="str">
-        <v>OpenLearn</v>
+        <v>Coursera</v>
       </c>
       <c r="E16" t="str">
-        <v>https://www.open.edu/openlearn/education-development/english-skills-learning</v>
+        <v>https://www.coursera.org/learn/business-writing</v>
       </c>
       <c r="F16" t="str">
         <v>Course</v>
@@ -1259,7 +1259,7 @@
         <v>Free</v>
       </c>
       <c r="I16" t="str">
-        <v>24 hours</v>
+        <v>13 hours</v>
       </c>
     </row>
     <row r="17">
@@ -1302,10 +1302,10 @@
         <v>Digital Storytelling</v>
       </c>
       <c r="D18" t="str">
-        <v>OpenLearn</v>
+        <v>Coursera</v>
       </c>
       <c r="E18" t="str">
-        <v>https://www.open.edu/openlearn/history-the-arts/digital-storytelling</v>
+        <v>https://www.coursera.org/learn/digital-storytelling</v>
       </c>
       <c r="F18" t="str">
         <v>Course</v>
@@ -1317,7 +1317,7 @@
         <v>Free</v>
       </c>
       <c r="I18" t="str">
-        <v>20 hours</v>
+        <v>16 hours</v>
       </c>
     </row>
     <row r="19">
@@ -1328,13 +1328,13 @@
         <v>S017</v>
       </c>
       <c r="C19" t="str">
-        <v>Intercultural Competence in the Workplace</v>
+        <v>Intercultural Communication and Conflict Resolution</v>
       </c>
       <c r="D19" t="str">
-        <v>OpenLearn</v>
+        <v>Coursera</v>
       </c>
       <c r="E19" t="str">
-        <v>https://www.open.edu/openlearn/languages/intercultural-competence-the-workplace</v>
+        <v>https://www.coursera.org/learn/intercultural-communication</v>
       </c>
       <c r="F19" t="str">
         <v>Course</v>
@@ -1346,7 +1346,7 @@
         <v>Free</v>
       </c>
       <c r="I19" t="str">
-        <v>12 hours</v>
+        <v>10 hours</v>
       </c>
     </row>
     <row r="20">
@@ -1360,10 +1360,10 @@
         <v>Business Ethics</v>
       </c>
       <c r="D20" t="str">
-        <v>OpenLearn</v>
+        <v>Coursera</v>
       </c>
       <c r="E20" t="str">
-        <v>https://www.open.edu/openlearn/money-business/business-ethics</v>
+        <v>https://www.coursera.org/learn/business-ethics</v>
       </c>
       <c r="F20" t="str">
         <v>Course</v>
@@ -1375,12 +1375,621 @@
         <v>Free</v>
       </c>
       <c r="I20" t="str">
-        <v>5 hours</v>
+        <v>8 hours</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>R020</v>
+      </c>
+      <c r="B21" t="str">
+        <v>S004</v>
+      </c>
+      <c r="C21" t="str">
+        <v>CS50: Introduction to Computer Science</v>
+      </c>
+      <c r="D21" t="str">
+        <v>edX / Harvard</v>
+      </c>
+      <c r="E21" t="str">
+        <v>https://www.edx.org/course/introduction-computer-science-harvardx-cs50x</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Course</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Beginner</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Free</v>
+      </c>
+      <c r="I21" t="str">
+        <v>12 weeks</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>R021</v>
+      </c>
+      <c r="B22" t="str">
+        <v>S004</v>
+      </c>
+      <c r="C22" t="str">
+        <v>100 Days of Code: The Complete Python Pro Bootcamp</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Udemy</v>
+      </c>
+      <c r="E22" t="str">
+        <v>https://www.udemy.com/course/100-days-of-code/</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Course</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Beginner</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="I22" t="str">
+        <v>60 hours</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>R022</v>
+      </c>
+      <c r="B23" t="str">
+        <v>S005</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Intro to Relational Databases</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Udacity</v>
+      </c>
+      <c r="E23" t="str">
+        <v>https://www.udacity.com/course/intro-to-relational-databases--ud197</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Course</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Intermediate</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Free</v>
+      </c>
+      <c r="I23" t="str">
+        <v>4 weeks</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>R023</v>
+      </c>
+      <c r="B24" t="str">
+        <v>S005</v>
+      </c>
+      <c r="C24" t="str">
+        <v>SQL Tutorial Full Database Course for Beginners</v>
+      </c>
+      <c r="D24" t="str">
+        <v>YouTube (freeCodeCamp)</v>
+      </c>
+      <c r="E24" t="str">
+        <v>https://www.youtube.com/watch?v=HXV3zeQKqGY</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Video</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Beginner</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Free</v>
+      </c>
+      <c r="I24" t="str">
+        <v>4 hours</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>R024</v>
+      </c>
+      <c r="B25" t="str">
+        <v>S001</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Communicating with Confidence</v>
+      </c>
+      <c r="D25" t="str">
+        <v>LinkedIn Learning</v>
+      </c>
+      <c r="E25" t="str">
+        <v>https://www.linkedin.com/learning/communicating-with-confidence</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Course</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Beginner</v>
+      </c>
+      <c r="H25" t="str">
+        <v>Subscription</v>
+      </c>
+      <c r="I25" t="str">
+        <v>1 hour</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>R025</v>
+      </c>
+      <c r="B26" t="str">
+        <v>S008</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Problem Solving (Basic)</v>
+      </c>
+      <c r="D26" t="str">
+        <v>HackerRank</v>
+      </c>
+      <c r="E26" t="str">
+        <v>https://www.hackerrank.com/skills-verification/problem_solving_basic</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Practice/Certification</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Beginner</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Free</v>
+      </c>
+      <c r="I26" t="str">
+        <v>Self-paced</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>R026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>S009</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Teamwork &amp; Collaboration</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Coursera</v>
+      </c>
+      <c r="E27" t="str">
+        <v>https://www.coursera.org/learn/leadership-collaboration</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Course</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Intermediate</v>
+      </c>
+      <c r="H27" t="str">
+        <v>Free</v>
+      </c>
+      <c r="I27" t="str">
+        <v>3 weeks</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>R027</v>
+      </c>
+      <c r="B28" t="str">
+        <v>S002</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Critical Thinking Masterclass</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Udemy</v>
+      </c>
+      <c r="E28" t="str">
+        <v>https://www.udemy.com/course/critical-thinking-masterclass/</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Course</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="H28" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="I28" t="str">
+        <v>2.5 hours</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>R028</v>
+      </c>
+      <c r="B29" t="str">
+        <v>S003</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Exercising Leadership: Foundational Principles</v>
+      </c>
+      <c r="D29" t="str">
+        <v>edX / Harvard</v>
+      </c>
+      <c r="E29" t="str">
+        <v>https://www.edx.org/course/exercising-leadership-foundational-principles</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Course</v>
+      </c>
+      <c r="G29" t="str">
+        <v>Beginner</v>
+      </c>
+      <c r="H29" t="str">
+        <v>Free</v>
+      </c>
+      <c r="I29" t="str">
+        <v>4 weeks</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>R029</v>
+      </c>
+      <c r="B30" t="str">
+        <v>S006</v>
+      </c>
+      <c r="C30" t="str">
+        <v>TED Masterclass: The Official Guide to Public Speaking</v>
+      </c>
+      <c r="D30" t="str">
+        <v>TED</v>
+      </c>
+      <c r="E30" t="str">
+        <v>https://masterclass.ted.com/</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Course</v>
+      </c>
+      <c r="G30" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="H30" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="I30" t="str">
+        <v>Self-paced</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>R030</v>
+      </c>
+      <c r="B31" t="str">
+        <v>S007</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Clinical Research</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Coursera</v>
+      </c>
+      <c r="E31" t="str">
+        <v>https://www.coursera.org/learn/clinical-research</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Course</v>
+      </c>
+      <c r="G31" t="str">
+        <v>Beginner</v>
+      </c>
+      <c r="H31" t="str">
+        <v>Free</v>
+      </c>
+      <c r="I31" t="str">
+        <v>3 weeks</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>R031</v>
+      </c>
+      <c r="B32" t="str">
+        <v>S010</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Ninja Writing: The Four Levels Of Writing Mastery</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Udemy</v>
+      </c>
+      <c r="E32" t="str">
+        <v>https://www.udemy.com/course/ninja-writing-the-four-levels-of-writing-mastery/</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Course</v>
+      </c>
+      <c r="G32" t="str">
+        <v>Intermediate</v>
+      </c>
+      <c r="H32" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="I32" t="str">
+        <v>4.5 hours</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>R032</v>
+      </c>
+      <c r="B33" t="str">
+        <v>S011</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Babbel Language Learning</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Babbel</v>
+      </c>
+      <c r="E33" t="str">
+        <v>https://www.babbel.com/</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Learning Platform</v>
+      </c>
+      <c r="G33" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Paid/Subscription</v>
+      </c>
+      <c r="I33" t="str">
+        <v>Self-paced</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>R033</v>
+      </c>
+      <c r="B34" t="str">
+        <v>S011</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Rosetta Stone</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Rosetta Stone</v>
+      </c>
+      <c r="E34" t="str">
+        <v>https://www.rosettastone.com/</v>
+      </c>
+      <c r="F34" t="str">
+        <v>Learning Platform</v>
+      </c>
+      <c r="G34" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="H34" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="I34" t="str">
+        <v>Self-paced</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>R034</v>
+      </c>
+      <c r="B35" t="str">
+        <v>S012</v>
+      </c>
+      <c r="C35" t="str">
+        <v>American Law</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Coursera</v>
+      </c>
+      <c r="E35" t="str">
+        <v>https://www.coursera.org/learn/american-law</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Course</v>
+      </c>
+      <c r="G35" t="str">
+        <v>Intermediate</v>
+      </c>
+      <c r="H35" t="str">
+        <v>Free</v>
+      </c>
+      <c r="I35" t="str">
+        <v>4 weeks</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>R035</v>
+      </c>
+      <c r="B36" t="str">
+        <v>S013</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Premiere Pro CC for Beginners: Video Editing in Premiere</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Udemy</v>
+      </c>
+      <c r="E36" t="str">
+        <v>https://www.udemy.com/course/adobe-premiere-pro-video-editing/</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Course</v>
+      </c>
+      <c r="G36" t="str">
+        <v>Beginner</v>
+      </c>
+      <c r="H36" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="I36" t="str">
+        <v>25 hours</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>R036</v>
+      </c>
+      <c r="B37" t="str">
+        <v>S014</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Data Analysis with R Programming</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Coursera / Google</v>
+      </c>
+      <c r="E37" t="str">
+        <v>https://www.coursera.org/learn/data-analysis-with-r</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Course</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Beginner</v>
+      </c>
+      <c r="H37" t="str">
+        <v>Free</v>
+      </c>
+      <c r="I37" t="str">
+        <v>36 hours</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>R037</v>
+      </c>
+      <c r="B38" t="str">
+        <v>S015</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Negotiation Skills</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Coursera</v>
+      </c>
+      <c r="E38" t="str">
+        <v>https://www.coursera.org/learn/negotiation-skills</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Course</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Intermediate</v>
+      </c>
+      <c r="H38" t="str">
+        <v>Free</v>
+      </c>
+      <c r="I38" t="str">
+        <v>4 weeks</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>R038</v>
+      </c>
+      <c r="B39" t="str">
+        <v>S016</v>
+      </c>
+      <c r="C39" t="str">
+        <v>QGIS for Beginners</v>
+      </c>
+      <c r="D39" t="str">
+        <v>YouTube (Klas Karlsson)</v>
+      </c>
+      <c r="E39" t="str">
+        <v>https://www.youtube.com/playlist?list=PL7MWEc0SRNQTQ4Hw6P_F9t2X-C4g-oQ3u</v>
+      </c>
+      <c r="F39" t="str">
+        <v>Playlist</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Beginner</v>
+      </c>
+      <c r="H39" t="str">
+        <v>Free</v>
+      </c>
+      <c r="I39" t="str">
+        <v>3 hours</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>R039</v>
+      </c>
+      <c r="B40" t="str">
+        <v>S017</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Intercultural Communication Courses</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Coursera</v>
+      </c>
+      <c r="E40" t="str">
+        <v>https://www.coursera.org/courses?query=intercultural+communication</v>
+      </c>
+      <c r="F40" t="str">
+        <v>Course Catalog</v>
+      </c>
+      <c r="G40" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="H40" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="I40" t="str">
+        <v>Variable</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>R040</v>
+      </c>
+      <c r="B41" t="str">
+        <v>S018</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Ethics in Action</v>
+      </c>
+      <c r="D41" t="str">
+        <v>edX / SDG Academy</v>
+      </c>
+      <c r="E41" t="str">
+        <v>https://www.edx.org/course/ethics-in-action</v>
+      </c>
+      <c r="F41" t="str">
+        <v>Course</v>
+      </c>
+      <c r="G41" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="H41" t="str">
+        <v>Free</v>
+      </c>
+      <c r="I41" t="str">
+        <v>6 weeks</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I41"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>